<commit_message>
9139 NE 10th Ave: no VersaShield (Marc)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_9139_NE_10th_Ave_TPO_Takeoff_Rev1.xlsx
+++ b/takeoffs/xlsx/2026-10-20_9139_NE_10th_Ave_TPO_Takeoff_Rev1.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1083,22 +1083,10 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VersaShield Solo slip sheet (only if fire rating requires)</t>
+          <t>Gutters (~124 LF) + 7 downspouts</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
-        <is>
-          <t>~5,100 SF</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Gutters (~124 LF) + 7 downspouts</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
         <is>
           <t>By others? confirm</t>
         </is>

</xml_diff>